<commit_message>
Count strength-modified ACMG codes in the agreement analysis
</commit_message>
<xml_diff>
--- a/figures/excel/Table_S9.xlsx
+++ b/figures/excel/Table_S9.xlsx
@@ -508,7 +508,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>0c9a22d44ff3eebe9b8edc2f5a58bf4b29f60184</t>
+          <t>53e183298613db292da35a4b45b1d3f6472cfbe8</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -873,7 +873,7 @@
     <row r="24" ht="34" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>NOTE: Generated on the machine that produced the deposit. DISCERN's own commit is the authoritative version: 0c9a22d44ff3eebe9b8edc2f5a58bf4b29f60184. Python package versions record the environment the committed results were produced in; continuous integration pins ruff and installs the remainder from pyproject.toml.</t>
+          <t>NOTE: Generated on the machine that produced the deposit. DISCERN's own commit is the authoritative version: 53e183298613db292da35a4b45b1d3f6472cfbe8. Python package versions record the environment the committed results were produced in; continuous integration pins ruff and installs the remainder from pyproject.toml.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Report the agreement denominator and correct the PM2 direction
</commit_message>
<xml_diff>
--- a/figures/excel/Table_S9.xlsx
+++ b/figures/excel/Table_S9.xlsx
@@ -508,7 +508,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>53e183298613db292da35a4b45b1d3f6472cfbe8</t>
+          <t>c500637f63aa48a01b8123b8299fc193801c4fe2</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -873,7 +873,7 @@
     <row r="24" ht="34" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>NOTE: Generated on the machine that produced the deposit. DISCERN's own commit is the authoritative version: 53e183298613db292da35a4b45b1d3f6472cfbe8. Python package versions record the environment the committed results were produced in; continuous integration pins ruff and installs the remainder from pyproject.toml.</t>
+          <t>NOTE: Generated on the machine that produced the deposit. DISCERN's own commit is the authoritative version: c500637f63aa48a01b8123b8299fc193801c4fe2. Python package versions record the environment the committed results were produced in; continuous integration pins ruff and installs the remainder from pyproject.toml.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Retarget the submission package and align the supplementary tables
</commit_message>
<xml_diff>
--- a/figures/excel/Table_S9.xlsx
+++ b/figures/excel/Table_S9.xlsx
@@ -508,7 +508,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>c500637f63aa48a01b8123b8299fc193801c4fe2</t>
+          <t>a15ad786a1584ee40737145087c7c31a18845164</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -873,7 +873,7 @@
     <row r="24" ht="34" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>NOTE: Generated on the machine that produced the deposit. DISCERN's own commit is the authoritative version: c500637f63aa48a01b8123b8299fc193801c4fe2. Python package versions record the environment the committed results were produced in; continuous integration pins ruff and installs the remainder from pyproject.toml.</t>
+          <t>NOTE: Generated on the machine that produced the deposit. DISCERN's own commit is the authoritative version: a15ad786a1584ee40737145087c7c31a18845164. Python package versions record the environment the committed results were produced in; continuous integration pins ruff and installs the remainder from pyproject.toml.</t>
         </is>
       </c>
     </row>

</xml_diff>